<commit_message>
itemData변경 / ItemType 분기
아이템 타입에 따른 인터페이스 작업
IActionItem
PlayerSight에서 분기
</commit_message>
<xml_diff>
--- a/Assets/02Script/Table/EscapeTable.xlsx
+++ b/Assets/02Script/Table/EscapeTable.xlsx
@@ -1,18 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GameSW\Documents\GitHub\EscapeRoom3D\Assets\02Script\Table\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E238A5-F9FE-4985-95F8-E44BC0864DF9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Object" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Dialogue" sheetId="2" r:id="rId5"/>
+    <sheet name="Object" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
   <si>
     <t>ItemID</t>
   </si>
@@ -35,7 +43,7 @@
     <t>PairID</t>
   </si>
   <si>
-    <t>DialogID</t>
+    <t>Dialog</t>
   </si>
   <si>
     <t>낡은 열쇠</t>
@@ -53,7 +61,7 @@
     <t>Pickable</t>
   </si>
   <si>
-    <t>장식용 책</t>
+    <t>None</t>
   </si>
   <si>
     <t>시험용 &lt;i&gt;책&lt;/i&gt;</t>
@@ -74,10 +82,7 @@
     <t>&lt;b&gt;무언가 허술한&lt;/b&gt; 자물쇠다.</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Interactive</t>
+    <t>Interactable</t>
   </si>
   <si>
     <t>낡은 일기</t>
@@ -92,54 +97,43 @@
     <t>Readable</t>
   </si>
   <si>
-    <t>Order</t>
-  </si>
-  <si>
-    <t>Text</t>
-  </si>
-  <si>
-    <t>시험용 일기. 25년 6월 23일</t>
-  </si>
-  <si>
-    <t>날씨가 꿀꿀하다</t>
-  </si>
-  <si>
-    <t>덥고 습하다</t>
-  </si>
-  <si>
-    <t>기
-분
-이
-별
-로</t>
-  </si>
-  <si>
-    <t>&lt;i&gt;좋다!!!&lt;/i&gt;</t>
-  </si>
-  <si>
-    <t>긴글 테스트. 동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세 동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세</t>
-  </si>
-  <si>
-    <t>긴글테스트2 동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세</t>
-  </si>
-  <si>
-    <t>다이얼로그 &lt;color=red&gt;끝!&lt;/color&gt;</t>
+    <t>긴글테스트2 동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세 
+다이얼로그 &lt;color=red&gt;끝!&lt;/color&gt;</t>
+  </si>
+  <si>
+    <t>안녕</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -148,40 +142,44 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -371,21 +369,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="22.5"/>
-    <col customWidth="1" min="4" max="4" width="27.88"/>
+    <col min="3" max="3" width="22.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.85546875" customWidth="1"/>
+    <col min="8" max="8" width="33.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -411,9 +413,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8">
       <c r="A2" s="1">
-        <v>1.0001001E7</v>
+        <v>10001001</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>8</v>
@@ -431,18 +433,18 @@
         <v>12</v>
       </c>
       <c r="G2" s="1">
-        <v>100.0</v>
-      </c>
-      <c r="H2" s="1">
-        <v>-1.0</v>
+        <v>100</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8">
       <c r="A3" s="1">
-        <v>1.0001002E7</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>10001002</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>14</v>
@@ -457,15 +459,15 @@
         <v>12</v>
       </c>
       <c r="G3" s="1">
-        <v>-1.0</v>
-      </c>
-      <c r="H3" s="1">
-        <v>-1.0</v>
+        <v>-1</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8">
       <c r="A4" s="1">
-        <v>2.0001001E7</v>
+        <v>20001001</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>17</v>
@@ -477,161 +479,47 @@
         <v>19</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1">
+        <v>100</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="1">
+        <v>30001001</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="1">
-        <v>100.0</v>
-      </c>
-      <c r="H4" s="1">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1">
-        <v>3.0001001E7</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="G5" s="1">
-        <v>-1.0</v>
-      </c>
-      <c r="H5" s="1">
-        <v>1.0</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="27.63"/>
-    <col customWidth="1" min="2" max="2" width="24.13"/>
-    <col customWidth="1" min="3" max="3" width="51.13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B2" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B4" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B5" s="1">
-        <v>3.0</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B6" s="1">
-        <v>4.0</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B7" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B8" s="1">
-        <v>6.0</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="B9" s="1">
-        <v>7.0</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Item구조 변경 + Room1
</commit_message>
<xml_diff>
--- a/Assets/02Script/Table/EscapeTable.xlsx
+++ b/Assets/02Script/Table/EscapeTable.xlsx
@@ -1,26 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GameSW\Documents\GitHub\EscapeRoom3D\Assets\02Script\Table\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E238A5-F9FE-4985-95F8-E44BC0864DF9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
-    <sheet name="Object" sheetId="1" r:id="rId1"/>
+    <sheet state="visible" name="Object" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
   <si>
     <t>ItemID</t>
   </si>
@@ -64,6 +55,9 @@
     <t>None</t>
   </si>
   <si>
+    <t>장식용 책</t>
+  </si>
+  <si>
     <t>시험용 &lt;i&gt;책&lt;/i&gt;</t>
   </si>
   <si>
@@ -83,6 +77,18 @@
   </si>
   <si>
     <t>Interactable</t>
+  </si>
+  <si>
+    <t>낡은 양동이</t>
+  </si>
+  <si>
+    <t>시험용 &lt;b&gt;양동이&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>&lt;i&gt;열리지 않은 이상한 양동이다.&lt;/i&gt;</t>
+  </si>
+  <si>
+    <t>Inspectable</t>
   </si>
   <si>
     <t>낡은 일기</t>
@@ -99,41 +105,22 @@
   <si>
     <t>긴글테스트2 동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세동해물과 백두산이 마르고닳도록 하느님이 보우하사 우리나라만세 무궁화 삼천리 화려강산 대한사람 대한으로 길이보전하세 
 다이얼로그 &lt;color=red&gt;끝!&lt;/color&gt;</t>
-  </si>
-  <si>
-    <t>안녕</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <fonts count="2">
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="3"/>
-      <charset val="129"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -142,44 +129,36 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="lightGray"/>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="2">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -369,25 +348,22 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col min="3" max="3" width="22.42578125" customWidth="1"/>
-    <col min="4" max="4" width="27.85546875" customWidth="1"/>
-    <col min="8" max="8" width="33.7109375" customWidth="1"/>
+    <col customWidth="1" min="3" max="3" width="22.5"/>
+    <col customWidth="1" min="4" max="4" width="27.88"/>
+    <col customWidth="1" min="8" max="8" width="33.75"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -413,9 +389,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2">
       <c r="A2" s="1">
-        <v>10001001</v>
+        <v>1.0001001E7</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>8</v>
@@ -433,93 +409,117 @@
         <v>12</v>
       </c>
       <c r="G2" s="1">
-        <v>100</v>
+        <v>100.0</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3">
       <c r="A3" s="1">
-        <v>10001002</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>1.0001002E7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="G3" s="1">
-        <v>-1</v>
+        <v>-1.0</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4">
       <c r="A4" s="1">
-        <v>20001001</v>
+        <v>2.0001001E7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" s="1">
-        <v>100</v>
+        <v>100.0</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5">
       <c r="A5" s="1">
-        <v>30001001</v>
+        <v>3.0001001E7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G5" s="1">
-        <v>-1</v>
+        <v>-1.0</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>25</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>4.0001001E7</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="1">
+        <v>-1.0</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>